<commit_message>
i18n(en): phase 2-4 — translate all content to English + reconcile cross-group tokens
Engine (scripts+tests), templates, potion example (incl. xlsx row4), methodology &
reference docs, 7 SKILL.md, and front-door docs translated to English. Load-bearing
tokens unified (manifest cols SystemID/Status/ModuleCode/Deps; status Draft/Playtesting/
Final/Recheck; config-spec Field/Type/Values/Range/Ref; DSL ## Skin/shape=circle/:observed;
Gherkin Feature/Scenario/Given/When/Then; aux files composite-key-map.json/ref-table-map.json/
enums.md). ref_lib RULE_RE gains (?![a-z]) so it won't carve R-M out of R-ModuleCode.
Verified: 0 residual CJK, 132 tests green, English example passes all 6 checkers.
</commit_message>
<xml_diff>
--- a/aigd/examples/potion-crafting/potion.xlsx
+++ b/aigd/examples/potion-crafting/potion.xlsx
@@ -483,27 +483,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>药水id</t>
+          <t>Potion id</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>名称文本id</t>
+          <t>Name text id</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>品质</t>
+          <t>Rarity</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>回血</t>
+          <t>Heal</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>合成消耗道具</t>
+          <t>Craft-cost item</t>
         </is>
       </c>
     </row>
@@ -633,17 +633,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>品质id</t>
+          <t>Rarity id</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>名称文本id</t>
+          <t>Name text id</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>叠加上限</t>
+          <t>Stack cap</t>
         </is>
       </c>
     </row>
@@ -728,12 +728,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>等级</t>
+          <t>Level</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>回血加成(累计)</t>
+          <t>Heal bonus (cumulative)</t>
         </is>
       </c>
     </row>
@@ -846,8 +846,6 @@
           <t>material[</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>]</t>
@@ -857,22 +855,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>配方id</t>
+          <t>Recipe id</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>产出药水</t>
+          <t>Output potion</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>材料药水</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>Material potion</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -887,8 +882,6 @@
       <c r="D5" t="n">
         <v>102</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -903,8 +896,6 @@
       <c r="D6" t="n">
         <v>101</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>